<commit_message>
fix: integer quest IDs and missing-link diagnostic
- Add to_int_id() mapping: RfD subquests 100.1–100.10 → integers 101–110;
  all quests originally numbered ≥101 shifted +10 to avoid collision.
  Eliminates decimal/float IDs in Excel and SAS tables.
- Apply to_int_id() to quest_id, from_id, and to_id in all output sheets.
- Warn at runtime when quests in quest_meta have no Lua block in api_raw.txt
  (currently 12 quests incl. Pandemonium whose prereqs are absent from the
  wiki's Module:Questreq/data — nodes are generated, edges are not).
- Regenerate quest_reference.xlsx and quest_network_sas.xlsx with new IDs.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/quest_reference.xlsx
+++ b/Data/quest_reference.xlsx
@@ -475,10 +475,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>178</t>
-        </is>
+      <c r="A2" t="n">
+        <v>188</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -506,10 +504,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="A3" t="n">
+        <v>0</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -537,10 +533,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>148</t>
-        </is>
+      <c r="A4" t="n">
+        <v>158</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -572,10 +566,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>142</t>
-        </is>
+      <c r="A5" t="n">
+        <v>152</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -603,10 +595,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>135</t>
-        </is>
+      <c r="A6" t="n">
+        <v>145</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -634,10 +624,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>129</t>
-        </is>
+      <c r="A7" t="n">
+        <v>139</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -665,10 +653,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
+      <c r="A8" t="n">
+        <v>51</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -696,10 +682,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
+      <c r="A9" t="n">
+        <v>17</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -731,10 +715,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="A10" t="n">
+        <v>16</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -762,10 +744,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="A11" t="n">
+        <v>15</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -793,10 +773,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
+      <c r="A12" t="n">
+        <v>14</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -828,10 +806,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="A13" t="n">
+        <v>13</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -859,10 +835,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="A14" t="n">
+        <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -894,10 +868,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+      <c r="A15" t="n">
+        <v>11</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -929,10 +901,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="A16" t="n">
+        <v>10</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -960,10 +930,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
+      <c r="A17" t="n">
+        <v>9</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -991,10 +959,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
+      <c r="A18" t="n">
+        <v>8</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1022,10 +988,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="A19" t="n">
+        <v>7</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1053,10 +1017,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="A20" t="n">
+        <v>3</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1084,10 +1046,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="A21" t="n">
+        <v>5</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1115,10 +1075,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="A22" t="n">
+        <v>6</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1146,10 +1104,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A23" t="n">
+        <v>2</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1177,10 +1133,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="A24" t="n">
+        <v>4</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1208,10 +1162,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A25" t="n">
+        <v>1</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1239,10 +1191,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+      <c r="A26" t="n">
+        <v>18</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1270,10 +1220,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
+      <c r="A27" t="n">
+        <v>19</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1305,10 +1253,8 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+      <c r="A28" t="n">
+        <v>20</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1336,10 +1282,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
+      <c r="A29" t="n">
+        <v>21</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1367,10 +1311,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
+      <c r="A30" t="n">
+        <v>22</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1406,10 +1348,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
+      <c r="A31" t="n">
+        <v>23</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1445,10 +1385,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+      <c r="A32" t="n">
+        <v>24</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1480,10 +1418,8 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
+      <c r="A33" t="n">
+        <v>26</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1515,10 +1451,8 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
+      <c r="A34" t="n">
+        <v>25</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1550,10 +1484,8 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
+      <c r="A35" t="n">
+        <v>27</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1581,10 +1513,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
+      <c r="A36" t="n">
+        <v>28</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1616,10 +1546,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="A37" t="n">
+        <v>29</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1647,10 +1575,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="A38" t="n">
+        <v>30</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1686,10 +1612,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
+      <c r="A39" t="n">
+        <v>31</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1717,10 +1641,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
+      <c r="A40" t="n">
+        <v>32</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1748,10 +1670,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
+      <c r="A41" t="n">
+        <v>33</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1779,10 +1699,8 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
+      <c r="A42" t="n">
+        <v>34</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1810,10 +1728,8 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="A43" t="n">
+        <v>35</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1841,10 +1757,8 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
+      <c r="A44" t="n">
+        <v>36</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1876,10 +1790,8 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
+      <c r="A45" t="n">
+        <v>37</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1907,10 +1819,8 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
+      <c r="A46" t="n">
+        <v>39</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -1946,10 +1856,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
+      <c r="A47" t="n">
+        <v>40</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -1981,10 +1889,8 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
+      <c r="A48" t="n">
+        <v>42</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -2020,10 +1926,8 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
+      <c r="A49" t="n">
+        <v>43</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -2051,10 +1955,8 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
+      <c r="A50" t="n">
+        <v>44</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -2086,10 +1988,8 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
+      <c r="A51" t="n">
+        <v>45</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -2125,10 +2025,8 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>46</t>
-        </is>
+      <c r="A52" t="n">
+        <v>46</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -2156,10 +2054,8 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
+      <c r="A53" t="n">
+        <v>47</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -2187,10 +2083,8 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
+      <c r="A54" t="n">
+        <v>48</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -2226,10 +2120,8 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
+      <c r="A55" t="n">
+        <v>49</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -2257,10 +2149,8 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+      <c r="A56" t="n">
+        <v>50</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -2296,10 +2186,8 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
+      <c r="A57" t="n">
+        <v>56</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -2327,10 +2215,8 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
+      <c r="A58" t="n">
+        <v>60</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -2366,10 +2252,8 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>52</t>
-        </is>
+      <c r="A59" t="n">
+        <v>52</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -2401,10 +2285,8 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
+      <c r="A60" t="n">
+        <v>53</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -2436,10 +2318,8 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
+      <c r="A61" t="n">
+        <v>55</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -2475,10 +2355,8 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>54</t>
-        </is>
+      <c r="A62" t="n">
+        <v>54</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -2506,10 +2384,8 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>59</t>
-        </is>
+      <c r="A63" t="n">
+        <v>59</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -2545,10 +2421,8 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>58</t>
-        </is>
+      <c r="A64" t="n">
+        <v>58</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -2584,10 +2458,8 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>57</t>
-        </is>
+      <c r="A65" t="n">
+        <v>57</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -2623,10 +2495,8 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
+      <c r="A66" t="n">
+        <v>61</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -2662,10 +2532,8 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>62</t>
-        </is>
+      <c r="A67" t="n">
+        <v>62</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -2693,10 +2561,8 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
+      <c r="A68" t="n">
+        <v>63</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -2732,10 +2598,8 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>64</t>
-        </is>
+      <c r="A69" t="n">
+        <v>64</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -2767,10 +2631,8 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
+      <c r="A70" t="n">
+        <v>65</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -2802,10 +2664,8 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>66</t>
-        </is>
+      <c r="A71" t="n">
+        <v>66</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -2841,10 +2701,8 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>67</t>
-        </is>
+      <c r="A72" t="n">
+        <v>67</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -2880,10 +2738,8 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
+      <c r="A73" t="n">
+        <v>68</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -2919,10 +2775,8 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>69</t>
-        </is>
+      <c r="A74" t="n">
+        <v>69</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -2958,10 +2812,8 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
+      <c r="A75" t="n">
+        <v>70</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -2997,10 +2849,8 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
+      <c r="A76" t="n">
+        <v>71</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -3036,10 +2886,8 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
+      <c r="A77" t="n">
+        <v>72</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -3075,10 +2923,8 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>73</t>
-        </is>
+      <c r="A78" t="n">
+        <v>73</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -3110,10 +2956,8 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>74</t>
-        </is>
+      <c r="A79" t="n">
+        <v>74</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -3149,10 +2993,8 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
+      <c r="A80" t="n">
+        <v>75</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -3184,10 +3026,8 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>76</t>
-        </is>
+      <c r="A81" t="n">
+        <v>76</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -3219,10 +3059,8 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>77</t>
-        </is>
+      <c r="A82" t="n">
+        <v>77</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -3258,10 +3096,8 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>78</t>
-        </is>
+      <c r="A83" t="n">
+        <v>78</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -3293,10 +3129,8 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>79</t>
-        </is>
+      <c r="A84" t="n">
+        <v>79</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -3328,10 +3162,8 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>81</t>
-        </is>
+      <c r="A85" t="n">
+        <v>81</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -3367,10 +3199,8 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>82</t>
-        </is>
+      <c r="A86" t="n">
+        <v>82</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -3402,10 +3232,8 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>83</t>
-        </is>
+      <c r="A87" t="n">
+        <v>83</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -3437,10 +3265,8 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
+      <c r="A88" t="n">
+        <v>84</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -3476,10 +3302,8 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>85</t>
-        </is>
+      <c r="A89" t="n">
+        <v>85</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -3515,10 +3339,8 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>86</t>
-        </is>
+      <c r="A90" t="n">
+        <v>86</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -3554,10 +3376,8 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>87</t>
-        </is>
+      <c r="A91" t="n">
+        <v>87</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -3589,10 +3409,8 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>88</t>
-        </is>
+      <c r="A92" t="n">
+        <v>88</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -3628,10 +3446,8 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
+      <c r="A93" t="n">
+        <v>89</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -3663,10 +3479,8 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
+      <c r="A94" t="n">
+        <v>90</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -3702,10 +3516,8 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
+      <c r="A95" t="n">
+        <v>91</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -3741,10 +3553,8 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>92</t>
-        </is>
+      <c r="A96" t="n">
+        <v>92</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -3776,10 +3586,8 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>93</t>
-        </is>
+      <c r="A97" t="n">
+        <v>93</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -3811,10 +3619,8 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>94</t>
-        </is>
+      <c r="A98" t="n">
+        <v>94</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -3846,10 +3652,8 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>95</t>
-        </is>
+      <c r="A99" t="n">
+        <v>95</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -3885,10 +3689,8 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>96</t>
-        </is>
+      <c r="A100" t="n">
+        <v>96</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -3920,10 +3722,8 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>97</t>
-        </is>
+      <c r="A101" t="n">
+        <v>97</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -3955,10 +3755,8 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>98</t>
-        </is>
+      <c r="A102" t="n">
+        <v>98</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -3994,10 +3792,8 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>99</t>
-        </is>
+      <c r="A103" t="n">
+        <v>99</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -4029,10 +3825,8 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="A104" t="n">
+        <v>100</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -4064,10 +3858,8 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>101</t>
-        </is>
+      <c r="A105" t="n">
+        <v>111</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -4103,10 +3895,8 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>102</t>
-        </is>
+      <c r="A106" t="n">
+        <v>112</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -4134,10 +3924,8 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>103</t>
-        </is>
+      <c r="A107" t="n">
+        <v>113</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -4165,10 +3953,8 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>104</t>
-        </is>
+      <c r="A108" t="n">
+        <v>114</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -4204,10 +3990,8 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>105</t>
-        </is>
+      <c r="A109" t="n">
+        <v>115</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -4243,10 +4027,8 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>106</t>
-        </is>
+      <c r="A110" t="n">
+        <v>116</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -4282,10 +4064,8 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>107</t>
-        </is>
+      <c r="A111" t="n">
+        <v>117</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -4321,10 +4101,8 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>108</t>
-        </is>
+      <c r="A112" t="n">
+        <v>118</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -4360,10 +4138,8 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>109</t>
-        </is>
+      <c r="A113" t="n">
+        <v>119</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -4399,10 +4175,8 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>110</t>
-        </is>
+      <c r="A114" t="n">
+        <v>120</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -4438,10 +4212,8 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>111</t>
-        </is>
+      <c r="A115" t="n">
+        <v>121</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -4477,10 +4249,8 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>112</t>
-        </is>
+      <c r="A116" t="n">
+        <v>122</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -4516,10 +4286,8 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>113</t>
-        </is>
+      <c r="A117" t="n">
+        <v>123</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -4555,10 +4323,8 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>114</t>
-        </is>
+      <c r="A118" t="n">
+        <v>124</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -4590,10 +4356,8 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>115</t>
-        </is>
+      <c r="A119" t="n">
+        <v>125</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -4625,10 +4389,8 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>116</t>
-        </is>
+      <c r="A120" t="n">
+        <v>126</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -4664,10 +4426,8 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>117</t>
-        </is>
+      <c r="A121" t="n">
+        <v>127</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -4699,10 +4459,8 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>118</t>
-        </is>
+      <c r="A122" t="n">
+        <v>128</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -4734,10 +4492,8 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>119</t>
-        </is>
+      <c r="A123" t="n">
+        <v>129</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -4773,10 +4529,8 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>121</t>
-        </is>
+      <c r="A124" t="n">
+        <v>131</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -4812,10 +4566,8 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>122</t>
-        </is>
+      <c r="A125" t="n">
+        <v>132</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -4851,10 +4603,8 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>123</t>
-        </is>
+      <c r="A126" t="n">
+        <v>133</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -4890,10 +4640,8 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
+      <c r="A127" t="n">
+        <v>134</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -4929,10 +4677,8 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>125</t>
-        </is>
+      <c r="A128" t="n">
+        <v>135</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -4968,10 +4714,8 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>126</t>
-        </is>
+      <c r="A129" t="n">
+        <v>136</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -5007,10 +4751,8 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>127</t>
-        </is>
+      <c r="A130" t="n">
+        <v>137</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -5046,10 +4788,8 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
+      <c r="A131" t="n">
+        <v>41</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -5085,10 +4825,8 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
+      <c r="A132" t="n">
+        <v>38</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -5120,10 +4858,8 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>120</t>
-        </is>
+      <c r="A133" t="n">
+        <v>130</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -5155,10 +4891,8 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>131</t>
-        </is>
+      <c r="A134" t="n">
+        <v>141</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -5194,10 +4928,8 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>151</t>
-        </is>
+      <c r="A135" t="n">
+        <v>161</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -5225,10 +4957,8 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
+      <c r="A136" t="n">
+        <v>175</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -5264,10 +4994,8 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
+      <c r="A137" t="n">
+        <v>80</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -5303,10 +5031,8 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>128</t>
-        </is>
+      <c r="A138" t="n">
+        <v>138</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -5342,10 +5068,8 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>130</t>
-        </is>
+      <c r="A139" t="n">
+        <v>140</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -5377,10 +5101,8 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>133</t>
-        </is>
+      <c r="A140" t="n">
+        <v>143</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -5416,10 +5138,8 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>132</t>
-        </is>
+      <c r="A141" t="n">
+        <v>142</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -5455,10 +5175,8 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>136</t>
-        </is>
+      <c r="A142" t="n">
+        <v>146</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -5494,10 +5212,8 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>134</t>
-        </is>
+      <c r="A143" t="n">
+        <v>144</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -5533,10 +5249,8 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>100.1</t>
-        </is>
+      <c r="A144" t="n">
+        <v>101</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -5572,10 +5286,8 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>100.3</t>
-        </is>
+      <c r="A145" t="n">
+        <v>103</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -5607,10 +5319,8 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>100.2</t>
-        </is>
+      <c r="A146" t="n">
+        <v>102</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -5642,10 +5352,8 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>100.6</t>
-        </is>
+      <c r="A147" t="n">
+        <v>106</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -5681,10 +5389,8 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>100.4</t>
-        </is>
+      <c r="A148" t="n">
+        <v>104</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -5720,10 +5426,8 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>100.5</t>
-        </is>
+      <c r="A149" t="n">
+        <v>105</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -5759,10 +5463,8 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>100.8</t>
-        </is>
+      <c r="A150" t="n">
+        <v>108</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -5798,10 +5500,8 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>100.7</t>
-        </is>
+      <c r="A151" t="n">
+        <v>107</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -5837,10 +5537,8 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>100.9</t>
-        </is>
+      <c r="A152" t="n">
+        <v>109</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -5876,10 +5574,8 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>138</t>
-        </is>
+      <c r="A153" t="n">
+        <v>148</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -5915,10 +5611,8 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>137</t>
-        </is>
+      <c r="A154" t="n">
+        <v>147</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -5954,10 +5648,8 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>139</t>
-        </is>
+      <c r="A155" t="n">
+        <v>149</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -5993,10 +5685,8 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>100.10</t>
-        </is>
+      <c r="A156" t="n">
+        <v>110</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -6032,10 +5722,8 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>143</t>
-        </is>
+      <c r="A157" t="n">
+        <v>153</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -6071,10 +5759,8 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>141</t>
-        </is>
+      <c r="A158" t="n">
+        <v>151</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -6110,10 +5796,8 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>140</t>
-        </is>
+      <c r="A159" t="n">
+        <v>150</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -6145,10 +5829,8 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>144</t>
-        </is>
+      <c r="A160" t="n">
+        <v>154</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -6184,10 +5866,8 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>170</t>
-        </is>
+      <c r="A161" t="n">
+        <v>180</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -6223,10 +5903,8 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>160</t>
-        </is>
+      <c r="A162" t="n">
+        <v>170</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -6262,10 +5940,8 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>145</t>
-        </is>
+      <c r="A163" t="n">
+        <v>155</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -6301,10 +5977,8 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+      <c r="A164" t="n">
+        <v>160</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -6340,10 +6014,8 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>146</t>
-        </is>
+      <c r="A165" t="n">
+        <v>156</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -6371,10 +6043,8 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>147</t>
-        </is>
+      <c r="A166" t="n">
+        <v>157</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -6406,10 +6076,8 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>149</t>
-        </is>
+      <c r="A167" t="n">
+        <v>159</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -6441,10 +6109,8 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>153</t>
-        </is>
+      <c r="A168" t="n">
+        <v>163</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -6472,10 +6138,8 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>152</t>
-        </is>
+      <c r="A169" t="n">
+        <v>162</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -6511,10 +6175,8 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>158</t>
-        </is>
+      <c r="A170" t="n">
+        <v>168</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -6550,10 +6212,8 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>154</t>
-        </is>
+      <c r="A171" t="n">
+        <v>164</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -6581,10 +6241,8 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>155</t>
-        </is>
+      <c r="A172" t="n">
+        <v>165</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -6616,10 +6274,8 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>157</t>
-        </is>
+      <c r="A173" t="n">
+        <v>167</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -6655,10 +6311,8 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>156</t>
-        </is>
+      <c r="A174" t="n">
+        <v>166</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -6694,10 +6348,8 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>159</t>
-        </is>
+      <c r="A175" t="n">
+        <v>169</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -6725,10 +6377,8 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>163</t>
-        </is>
+      <c r="A176" t="n">
+        <v>173</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -6764,10 +6414,8 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>164</t>
-        </is>
+      <c r="A177" t="n">
+        <v>174</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -6803,10 +6451,8 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>161</t>
-        </is>
+      <c r="A178" t="n">
+        <v>171</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -6838,10 +6484,8 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>162</t>
-        </is>
+      <c r="A179" t="n">
+        <v>172</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -6877,10 +6521,8 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>166</t>
-        </is>
+      <c r="A180" t="n">
+        <v>176</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -6916,10 +6558,8 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>167</t>
-        </is>
+      <c r="A181" t="n">
+        <v>177</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -6955,10 +6595,8 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>168</t>
-        </is>
+      <c r="A182" t="n">
+        <v>178</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -6990,10 +6628,8 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>169</t>
-        </is>
+      <c r="A183" t="n">
+        <v>179</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -7029,10 +6665,8 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>171</t>
-        </is>
+      <c r="A184" t="n">
+        <v>181</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -7060,10 +6694,8 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>174</t>
-        </is>
+      <c r="A185" t="n">
+        <v>184</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -7091,10 +6723,8 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>175</t>
-        </is>
+      <c r="A186" t="n">
+        <v>185</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -7122,10 +6752,8 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>176</t>
-        </is>
+      <c r="A187" t="n">
+        <v>186</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -7153,10 +6781,8 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>177</t>
-        </is>
+      <c r="A188" t="n">
+        <v>187</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -7184,10 +6810,8 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>172</t>
-        </is>
+      <c r="A189" t="n">
+        <v>182</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -7215,10 +6839,8 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>173</t>
-        </is>
+      <c r="A190" t="n">
+        <v>183</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>

</xml_diff>